<commit_message>
Reconcile new Azbil diagrams; add DHW/sanitary/filtration/smoke + comms model
Reconcile 7 supplied Azbil PDFs (central-monitoring hardware spec, comms trunk,
instrumentation, live BMS summary screens) against the model. Extend the
functional model with four supervised subsystems surfaced by the BMS graphics —
domestic hot water, plumbing/sanitary, recreational-water filtration, smoke
control — plus CO2 DCV on banquet AHUs, and add a Comms-Network sheet capturing
the savic-netFX2 central + 6-SCS/NC-bus/RS fieldbus architecture. Model grows
1,160->1,383 pts, 190->259 devices, 12->16 panels, 84->109 DDC controllers;
SOO + GCL+ + exports regenerated. See docs/reconciliation_2026-08.md.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/exports/red5-dhcp_electrical.xlsx
+++ b/exports/red5-dhcp_electrical.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Flat" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Flat'!$A$1:$J$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Flat'!$A$1:$J$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -517,7 +517,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Generated 2026-07-30  ·  source: generate_io_list.py</t>
+          <t>Generated 2026-08-03  ·  source: generate_io_list.py</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
@@ -548,7 +548,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>60</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8">
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>62</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10">
@@ -786,17 +786,17 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>LCP-4F</t>
+          <t>LCP-2F</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>4F–5F air-side panel</t>
+          <t>2F air-side panel</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>4F AHU Room</t>
+          <t>2F AHU Room</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
@@ -821,63 +821,133 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>LCP-PKG</t>
+          <t>LCP-4F</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Packaged-unit &amp; refrigeration panel</t>
+          <t>4F–5F air-side panel</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>B3F–B1F EPS</t>
+          <t>4F AHU Room</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>LCP-PKG</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Packaged-unit &amp; refrigeration panel</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>B3F–B1F EPS</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="I17" s="4" t="n">
+      <c r="I18" s="4" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>B3F–B2F plant</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr"/>
-      <c r="C18" s="5" t="inlineStr"/>
-      <c r="D18" s="5" t="n">
-        <v>26</v>
-      </c>
-      <c r="E18" s="5" t="n">
+      <c r="B20" s="5" t="inlineStr"/>
+      <c r="C20" s="5" t="inlineStr"/>
+      <c r="D20" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="E20" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="F18" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="H18" s="5" t="n">
+      <c r="F20" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="H20" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="I18" s="5" t="n">
-        <v>62</v>
+      <c r="I20" s="5" t="n">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -891,7 +961,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3081,12 +3151,12 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>LCP-4F</t>
+          <t>LCP-2F</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>4F–5F air-side panel</t>
+          <t>2F air-side panel</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr"/>
@@ -3097,12 +3167,12 @@
     <row r="84" outlineLevel="1">
       <c r="A84" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    DDC-4F-03</t>
+          <t xml:space="preserve">    DDC-2F-02</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>EVU-8, EVU-9, EVU-10</t>
+          <t>AC-11, AC-12, AC-13</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr"/>
@@ -3113,17 +3183,17 @@
     <row r="85" outlineLevel="2">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        EVU-8.SPD</t>
+          <t xml:space="preserve">        AC-11.OAD</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Supply fan VFD (INV) speed</t>
+          <t>Outdoor-air damper</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>EVU-8</t>
+          <t>AC-11</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -3145,17 +3215,17 @@
     <row r="86" outlineLevel="2">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        EVU-9.SPD</t>
+          <t xml:space="preserve">        AC-12.OAD</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Supply fan VFD (INV) speed</t>
+          <t>Outdoor-air damper</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>EVU-9</t>
+          <t>AC-12</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -3177,17 +3247,17 @@
     <row r="87" outlineLevel="2">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        EVU-10.SPD</t>
+          <t xml:space="preserve">        AC-13.OAD</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Supply fan VFD (INV) speed</t>
+          <t>Outdoor-air damper</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>EVU-10</t>
+          <t>AC-13</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -3209,12 +3279,12 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>LCP-PKG</t>
+          <t>LCP-4F</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Packaged-unit &amp; refrigeration panel</t>
+          <t>4F–5F air-side panel</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr"/>
@@ -3225,12 +3295,12 @@
     <row r="89" outlineLevel="1">
       <c r="A89" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    DDC-PKG-01</t>
+          <t xml:space="preserve">    DDC-4F-03</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>PAC-1-1, PAC-1-2, PAC-2</t>
+          <t>EVU-8, EVU-9, EVU-10</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr"/>
@@ -3241,151 +3311,135 @@
     <row r="90" outlineLevel="2">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PAC-1-1.SS</t>
+          <t xml:space="preserve">        EVU-8.SPD</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Start/Stop command</t>
+          <t>Supply fan VFD (INV) speed</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>PAC-1-1</t>
+          <t>EVU-8</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>AO</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>Packaged units</t>
+          <t>Air side</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>%</t>
         </is>
       </c>
     </row>
     <row r="91" outlineLevel="2">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PAC-1-2.SS</t>
+          <t xml:space="preserve">        EVU-9.SPD</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Start/Stop command</t>
+          <t>Supply fan VFD (INV) speed</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>PAC-1-2</t>
+          <t>EVU-9</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>AO</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>Packaged units</t>
+          <t>Air side</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>%</t>
         </is>
       </c>
     </row>
     <row r="92" outlineLevel="2">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PAC-2.SS</t>
+          <t xml:space="preserve">        EVU-10.SPD</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Start/Stop command</t>
+          <t>Supply fan VFD (INV) speed</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>PAC-2</t>
+          <t>EVU-10</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>AO</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>Packaged units</t>
+          <t>Air side</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" outlineLevel="1">
-      <c r="A93" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    DDC-PKG-02</t>
-        </is>
-      </c>
-      <c r="B93" s="7" t="inlineStr">
-        <is>
-          <t>PAC-3, PAC-4, PAC-5</t>
-        </is>
-      </c>
-      <c r="C93" s="7" t="inlineStr"/>
-      <c r="D93" s="7" t="inlineStr"/>
-      <c r="E93" s="7" t="inlineStr"/>
-      <c r="F93" s="7" t="inlineStr"/>
-    </row>
-    <row r="94" outlineLevel="2">
-      <c r="A94" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        PAC-3.SS</t>
-        </is>
-      </c>
-      <c r="B94" s="4" t="inlineStr">
-        <is>
-          <t>Start/Stop command</t>
-        </is>
-      </c>
-      <c r="C94" s="4" t="inlineStr">
-        <is>
-          <t>PAC-3</t>
-        </is>
-      </c>
-      <c r="D94" s="4" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="E94" s="4" t="inlineStr">
-        <is>
-          <t>Packaged units</t>
-        </is>
-      </c>
-      <c r="F94" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>LCP-PKG</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Packaged-unit &amp; refrigeration panel</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr"/>
+      <c r="D93" s="5" t="inlineStr"/>
+      <c r="E93" s="5" t="inlineStr"/>
+      <c r="F93" s="5" t="inlineStr"/>
+    </row>
+    <row r="94" outlineLevel="1">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DDC-PKG-01</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>PAC-1-1, PAC-1-2, PAC-2</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr"/>
+      <c r="D94" s="7" t="inlineStr"/>
+      <c r="E94" s="7" t="inlineStr"/>
+      <c r="F94" s="7" t="inlineStr"/>
     </row>
     <row r="95" outlineLevel="2">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PAC-4.SS</t>
+          <t xml:space="preserve">        PAC-1-1.SS</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
@@ -3395,7 +3449,7 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>PAC-4</t>
+          <t>PAC-1-1</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -3417,30 +3471,814 @@
     <row r="96" outlineLevel="2">
       <c r="A96" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">        PAC-1-2.SS</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Start/Stop command</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>PAC-1-2</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>Packaged units</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" outlineLevel="2">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        PAC-2.SS</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>Start/Stop command</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>PAC-2</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>Packaged units</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" outlineLevel="1">
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DDC-PKG-02</t>
+        </is>
+      </c>
+      <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>PAC-3, PAC-4, PAC-5</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr"/>
+      <c r="D98" s="7" t="inlineStr"/>
+      <c r="E98" s="7" t="inlineStr"/>
+      <c r="F98" s="7" t="inlineStr"/>
+    </row>
+    <row r="99" outlineLevel="2">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        PAC-3.SS</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>Start/Stop command</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>PAC-3</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>Packaged units</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" outlineLevel="2">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        PAC-4.SS</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Start/Stop command</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>PAC-4</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>Packaged units</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" outlineLevel="2">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">        PAC-5.SS</t>
         </is>
       </c>
-      <c r="B96" s="4" t="inlineStr">
+      <c r="B101" s="4" t="inlineStr">
         <is>
           <t>Start/Stop command</t>
         </is>
       </c>
-      <c r="C96" s="4" t="inlineStr">
+      <c r="C101" s="4" t="inlineStr">
         <is>
           <t>PAC-5</t>
         </is>
       </c>
-      <c r="D96" s="4" t="inlineStr">
+      <c r="D101" s="4" t="inlineStr">
         <is>
           <t>BO</t>
         </is>
       </c>
-      <c r="E96" s="4" t="inlineStr">
+      <c r="E101" s="4" t="inlineStr">
         <is>
           <t>Packaged units</t>
         </is>
       </c>
-      <c r="F96" s="4" t="inlineStr">
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr"/>
+      <c r="D102" s="5" t="inlineStr"/>
+      <c r="E102" s="5" t="inlineStr"/>
+      <c r="F102" s="5" t="inlineStr"/>
+    </row>
+    <row r="103" outlineLevel="1">
+      <c r="A103" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DDC-SAN-01</t>
+        </is>
+      </c>
+      <c r="B103" s="7" t="inlineStr">
+        <is>
+          <t>MP-1, MP-2, MP-3</t>
+        </is>
+      </c>
+      <c r="C103" s="7" t="inlineStr"/>
+      <c r="D103" s="7" t="inlineStr"/>
+      <c r="E103" s="7" t="inlineStr"/>
+      <c r="F103" s="7" t="inlineStr"/>
+    </row>
+    <row r="104" outlineLevel="2">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        MP-1.TRIP</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>MP-1</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" outlineLevel="2">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        MP-2.TRIP</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>MP-2</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" outlineLevel="2">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        MP-3.TRIP</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>MP-3</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F106" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" outlineLevel="1">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DDC-SAN-02</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>MP-4, P-1, P-2</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="inlineStr"/>
+      <c r="D107" s="7" t="inlineStr"/>
+      <c r="E107" s="7" t="inlineStr"/>
+      <c r="F107" s="7" t="inlineStr"/>
+    </row>
+    <row r="108" outlineLevel="2">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        MP-4.TRIP</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C108" s="4" t="inlineStr">
+        <is>
+          <t>MP-4</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" outlineLevel="2">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        P-1.TRIP</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>P-1</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F109" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" outlineLevel="2">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        P-2.TRIP</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>P-2</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" outlineLevel="1">
+      <c r="A111" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DDC-SAN-03</t>
+        </is>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>P-3, P-4, P-5</t>
+        </is>
+      </c>
+      <c r="C111" s="7" t="inlineStr"/>
+      <c r="D111" s="7" t="inlineStr"/>
+      <c r="E111" s="7" t="inlineStr"/>
+      <c r="F111" s="7" t="inlineStr"/>
+    </row>
+    <row r="112" outlineLevel="2">
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        P-3.TRIP</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>P-3</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F112" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" outlineLevel="2">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        P-4.TRIP</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>P-4</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F113" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" outlineLevel="2">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        P-5.TRIP</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C114" s="4" t="inlineStr">
+        <is>
+          <t>P-5</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F114" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" outlineLevel="1">
+      <c r="A115" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DDC-SAN-04</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>P-6, RCVT-1, ELVT-1</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr"/>
+      <c r="D115" s="7" t="inlineStr"/>
+      <c r="E115" s="7" t="inlineStr"/>
+      <c r="F115" s="7" t="inlineStr"/>
+    </row>
+    <row r="116" outlineLevel="2">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        P-6.TRIP</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>P-6</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F116" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" outlineLevel="1">
+      <c r="A117" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DDC-SAN-10</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>DP-14, BL-1-1, BL-1-2</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr"/>
+      <c r="D117" s="7" t="inlineStr"/>
+      <c r="E117" s="7" t="inlineStr"/>
+      <c r="F117" s="7" t="inlineStr"/>
+    </row>
+    <row r="118" outlineLevel="2">
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        BL-1-1.TRIP</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>BL-1-1</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F118" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" outlineLevel="2">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        BL-1-2.TRIP</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>BL-1-2</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F119" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" outlineLevel="1">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DDC-SAN-11</t>
+        </is>
+      </c>
+      <c r="B120" s="7" t="inlineStr">
+        <is>
+          <t>BL-2-1, BL-2-2, BL-F-1</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr"/>
+      <c r="D120" s="7" t="inlineStr"/>
+      <c r="E120" s="7" t="inlineStr"/>
+      <c r="F120" s="7" t="inlineStr"/>
+    </row>
+    <row r="121" outlineLevel="2">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        BL-2-1.TRIP</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>BL-2-1</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" outlineLevel="2">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        BL-2-2.TRIP</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>BL-2-2</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" outlineLevel="2">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        BL-F-1.TRIP</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>BL-F-1</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F123" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" outlineLevel="1">
+      <c r="A124" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DDC-SAN-12</t>
+        </is>
+      </c>
+      <c r="B124" s="7" t="inlineStr">
+        <is>
+          <t>BL-F-2</t>
+        </is>
+      </c>
+      <c r="C124" s="7" t="inlineStr"/>
+      <c r="D124" s="7" t="inlineStr"/>
+      <c r="E124" s="7" t="inlineStr"/>
+      <c r="F124" s="7" t="inlineStr"/>
+    </row>
+    <row r="125" outlineLevel="2">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        BL-F-2.TRIP</t>
+        </is>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>BL-F-2</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="F125" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3457,7 +4295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6127,27 +6965,27 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>LCP-4F</t>
+          <t>LCP-2F</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>4F–5F air-side panel</t>
+          <t>2F air-side panel</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>DDC-4F-03</t>
+          <t>DDC-2F-02</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>EVU-8</t>
+          <t>AC-11</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>EVU-8.SPD</t>
+          <t>AC-11.OAD</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -6167,39 +7005,39 @@
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>Supply fan VFD (INV) speed</t>
+          <t>Outdoor-air damper</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
-          <t>INV schedule; demand vent</t>
+          <t>CO2 demand-controlled reset (DCV)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>LCP-4F</t>
+          <t>LCP-2F</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>4F–5F air-side panel</t>
+          <t>2F air-side panel</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>DDC-4F-03</t>
+          <t>DDC-2F-02</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>EVU-9</t>
+          <t>AC-12</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>EVU-9.SPD</t>
+          <t>AC-12.OAD</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
@@ -6219,39 +7057,39 @@
       </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>Supply fan VFD (INV) speed</t>
+          <t>Outdoor-air damper</t>
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
-          <t>INV schedule; demand vent</t>
+          <t>CO2 demand-controlled reset (DCV)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>LCP-4F</t>
+          <t>LCP-2F</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>4F–5F air-side panel</t>
+          <t>2F air-side panel</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>DDC-4F-03</t>
+          <t>DDC-2F-02</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>EVU-10</t>
+          <t>AC-13</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>EVU-10.SPD</t>
+          <t>AC-13.OAD</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -6271,168 +7109,168 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>Supply fan VFD (INV) speed</t>
+          <t>Outdoor-air damper</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
-          <t>INV schedule; demand vent</t>
+          <t>CO2 demand-controlled reset (DCV)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>LCP-PKG</t>
+          <t>LCP-4F</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Packaged-unit &amp; refrigeration panel</t>
+          <t>4F–5F air-side panel</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>DDC-PKG-01</t>
+          <t>DDC-4F-03</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>PAC-1-1</t>
+          <t>EVU-8</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>PAC-1-1.SS</t>
+          <t>EVU-8.SPD</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>AO</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>Packaged units</t>
+          <t>Air side</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>%</t>
         </is>
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>Start/Stop command</t>
+          <t>Supply fan VFD (INV) speed</t>
         </is>
       </c>
       <c r="J58" s="4" t="inlineStr">
         <is>
-          <t>24/7 (electrical room)</t>
+          <t>INV schedule; demand vent</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>LCP-PKG</t>
+          <t>LCP-4F</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Packaged-unit &amp; refrigeration panel</t>
+          <t>4F–5F air-side panel</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>DDC-PKG-01</t>
+          <t>DDC-4F-03</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>PAC-1-2</t>
+          <t>EVU-9</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>PAC-1-2.SS</t>
+          <t>EVU-9.SPD</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>AO</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>Packaged units</t>
+          <t>Air side</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>%</t>
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>Start/Stop command</t>
+          <t>Supply fan VFD (INV) speed</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
         <is>
-          <t>24/7 (electrical room)</t>
+          <t>INV schedule; demand vent</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>LCP-PKG</t>
+          <t>LCP-4F</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Packaged-unit &amp; refrigeration panel</t>
+          <t>4F–5F air-side panel</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>DDC-PKG-01</t>
+          <t>DDC-4F-03</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>PAC-2</t>
+          <t>EVU-10</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>PAC-2.SS</t>
+          <t>EVU-10.SPD</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>AO</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>Packaged units</t>
+          <t>Air side</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>%</t>
         </is>
       </c>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>Start/Stop command</t>
+          <t>Supply fan VFD (INV) speed</t>
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
-          <t>24/7 (electrical room)</t>
+          <t>INV schedule; demand vent</t>
         </is>
       </c>
     </row>
@@ -6449,17 +7287,17 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>DDC-PKG-02</t>
+          <t>DDC-PKG-01</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>PAC-3</t>
+          <t>PAC-1-1</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>PAC-3.SS</t>
+          <t>PAC-1-1.SS</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -6501,17 +7339,17 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>DDC-PKG-02</t>
+          <t>DDC-PKG-01</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>PAC-4</t>
+          <t>PAC-1-2</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>PAC-4.SS</t>
+          <t>PAC-1-2.SS</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
@@ -6553,47 +7391,971 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
+          <t>DDC-PKG-01</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>PAC-2</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>PAC-2.SS</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>Packaged units</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>Start/Stop command</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>24/7 (electrical room)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>LCP-PKG</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Packaged-unit &amp; refrigeration panel</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
           <t>DDC-PKG-02</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>PAC-3</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>PAC-3.SS</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>Packaged units</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>Start/Stop command</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>24/7 (electrical room)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>LCP-PKG</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Packaged-unit &amp; refrigeration panel</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>DDC-PKG-02</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>PAC-4</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>PAC-4.SS</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>Packaged units</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>Start/Stop command</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>24/7 (electrical room)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>LCP-PKG</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Packaged-unit &amp; refrigeration panel</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>DDC-PKG-02</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
         <is>
           <t>PAC-5</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="E66" s="4" t="inlineStr">
         <is>
           <t>PAC-5.SS</t>
         </is>
       </c>
-      <c r="F63" s="4" t="inlineStr">
+      <c r="F66" s="4" t="inlineStr">
         <is>
           <t>BO</t>
         </is>
       </c>
-      <c r="G63" s="4" t="inlineStr">
+      <c r="G66" s="4" t="inlineStr">
         <is>
           <t>Packaged units</t>
         </is>
       </c>
-      <c r="H63" s="4" t="inlineStr">
+      <c r="H66" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I63" s="4" t="inlineStr">
+      <c r="I66" s="4" t="inlineStr">
         <is>
           <t>Start/Stop command</t>
         </is>
       </c>
-      <c r="J63" s="4" t="inlineStr">
+      <c r="J66" s="4" t="inlineStr">
         <is>
           <t>24/7 (electrical room)</t>
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-01</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>MP-1</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>MP-1.TRIP</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-01</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>MP-2</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>MP-2.TRIP</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-01</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>MP-3</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>MP-3.TRIP</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-02</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>MP-4</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>MP-4.TRIP</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-02</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>P-1</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>P-1.TRIP</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-02</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>P-2</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>P-2.TRIP</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-03</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>P-3</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>P-3.TRIP</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-03</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>P-4</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>P-4.TRIP</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-03</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>P-5</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>P-5.TRIP</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-04</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>P-6</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>P-6.TRIP</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-10</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>BL-1-1</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>BL-1-1.TRIP</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-10</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>BL-1-2</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>BL-1-2.TRIP</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-11</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>BL-2-1</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>BL-2-1.TRIP</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-11</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>BL-2-2</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>BL-2-2.TRIP</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-11</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>BL-F-1</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>BL-F-1.TRIP</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>LCP-SAN</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing / sanitary panel (上水・中水・排水)</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>DDC-SAN-12</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>BL-F-2</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>BL-F-2.TRIP</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing/Sanitary</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>Pump fault / breaker trip</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J63"/>
+  <autoFilter ref="A1:J82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>